<commit_message>
fix #REF! in Netherlands_data sheet
</commit_message>
<xml_diff>
--- a/vignettes/CaseStudies/LEON-T/Microplastic_variables_v1.1c.xlsx
+++ b/vignettes/CaseStudies/LEON-T/Microplastic_variables_v1.1c.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{204F37EE-04D1-45C6-8599-07F7F6020AB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E2C9F70-A795-4175-8A11-95CE2671FD21}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC4F2E84-D90A-4D6B-8DCE-3898256B3B03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13410" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="19" r:id="rId1"/>
@@ -16,6 +16,9 @@
     <sheet name="Tables" sheetId="20" r:id="rId6"/>
     <sheet name="TRWP_data" sheetId="21" r:id="rId7"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId8"/>
+  </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Polymer_data!$A$1:$T$60</definedName>
   </definedNames>
@@ -787,7 +790,7 @@
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -866,7 +869,6 @@
     <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="40% - Accent3" xfId="3" builtinId="39"/>
@@ -891,12 +893,76 @@
 </styleSheet>
 </file>
 
-<file path=xl/namedSheetViews/namedSheetView1.xml><?xml version="1.0" encoding="utf-8"?>
-<namedSheetViews xmlns="http://schemas.microsoft.com/office/spreadsheetml/2019/namedsheetviews" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="About"/>
+      <sheetName val="Polymer_data"/>
+      <sheetName val="Correlation"/>
+      <sheetName val="Netherlands_data"/>
+      <sheetName val="Distributions"/>
+      <sheetName val="Variables"/>
+      <sheetName val="Tables"/>
+      <sheetName val="Variables to implement"/>
+      <sheetName val="TRWP_data"/>
+      <sheetName val="Trapezoidal distributions"/>
+      <sheetName val="Rubber notes"/>
+      <sheetName val="Road side soil area"/>
+      <sheetName val="Netherlands scale calculations"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12">
+        <row r="2">
+          <cell r="C2">
+            <v>9.9944635678694368E-2</v>
+          </cell>
+          <cell r="H2">
+            <v>0.5965071808724024</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="H3">
+            <v>5.3060897007301225E-2</v>
+          </cell>
+        </row>
+        <row r="4">
+          <cell r="B4">
+            <v>41543</v>
+          </cell>
+          <cell r="H4">
+            <v>0.13412318472359658</v>
+          </cell>
+        </row>
+        <row r="5">
+          <cell r="H5">
+            <v>0.16923858682570672</v>
+          </cell>
+        </row>
+        <row r="6">
+          <cell r="H6">
+            <v>4.7070150570993022E-2</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1404,15 +1470,15 @@
         <v>1</v>
       </c>
       <c r="O3" s="6" t="b">
-        <f>I3&gt;J3</f>
+        <f t="shared" ref="O3:O26" si="1">I3&gt;J3</f>
         <v>1</v>
       </c>
       <c r="P3" s="11">
-        <f t="shared" ref="P3:Q4" si="1">H3*3600*24</f>
+        <f t="shared" ref="P3:Q4" si="2">H3*3600*24</f>
         <v>8.6400000000000004E-16</v>
       </c>
       <c r="Q3" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.7280000000000003E-4</v>
       </c>
       <c r="R3" s="11">
@@ -1457,15 +1523,15 @@
         <v>1</v>
       </c>
       <c r="O4" s="6" t="b">
-        <f>I4&gt;J4</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P4" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>8.6400000000000004E-16</v>
       </c>
       <c r="Q4" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>8.6400000000000013E-5</v>
       </c>
       <c r="R4" s="11">
@@ -1503,11 +1569,11 @@
         <v>20</v>
       </c>
       <c r="N5" s="6" t="b">
-        <f>I5&gt;H5</f>
+        <f t="shared" ref="N5:N14" si="3">I5&gt;H5</f>
         <v>1</v>
       </c>
       <c r="O5" s="6" t="b">
-        <f>I5&gt;J5</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P5" s="6"/>
@@ -1547,11 +1613,11 @@
         <v>20</v>
       </c>
       <c r="N6" s="6" t="b">
-        <f>I6&gt;H6</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O6" s="6" t="b">
-        <f>I6&gt;J6</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P6" s="6"/>
@@ -1594,17 +1660,17 @@
         <v>39</v>
       </c>
       <c r="N7" s="6" t="b">
-        <f>I7&gt;H7</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O7" s="6" t="b">
-        <f>I7&gt;J7</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P7" s="6"/>
       <c r="Q7" s="6"/>
       <c r="R7" s="11">
-        <f t="shared" ref="R7:R16" si="2">J7*3600*24</f>
+        <f t="shared" ref="R7:R16" si="4">J7*3600*24</f>
         <v>2.3328000000000003E-3</v>
       </c>
       <c r="S7" s="11"/>
@@ -1640,17 +1706,17 @@
         <v>20</v>
       </c>
       <c r="N8" s="6" t="b">
-        <f>I8&gt;H8</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O8" s="6" t="b">
-        <f>I8&gt;J8</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P8" s="6"/>
       <c r="Q8" s="6"/>
       <c r="R8" s="11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S8" s="11"/>
@@ -1694,17 +1760,17 @@
         <v>27</v>
       </c>
       <c r="N9" s="6" t="b">
-        <f>I9&gt;H9</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O9" s="6" t="b">
-        <f>I9&gt;J9</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P9" s="6"/>
       <c r="Q9" s="6"/>
       <c r="R9" s="11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2.3800000000000004E-4</v>
       </c>
       <c r="S9" s="11"/>
@@ -1746,17 +1812,17 @@
         <v>45</v>
       </c>
       <c r="N10" s="6" t="b">
-        <f>I10&gt;H10</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O10" s="6" t="b">
-        <f>I10&gt;J10</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P10" s="6"/>
       <c r="Q10" s="6"/>
       <c r="R10" s="11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S10" s="11"/>
@@ -1799,23 +1865,23 @@
         <v>27</v>
       </c>
       <c r="N11" s="6" t="b">
-        <f>I11&gt;H11</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O11" s="6" t="b">
-        <f>I11&gt;J11</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P11" s="11">
-        <f t="shared" ref="P11" si="3">H11*3600*24</f>
+        <f t="shared" ref="P11" si="5">H11*3600*24</f>
         <v>2E-3</v>
       </c>
       <c r="Q11" s="11">
-        <f t="shared" ref="Q11" si="4">I11*3600*24</f>
+        <f t="shared" ref="Q11" si="6">I11*3600*24</f>
         <v>2.6999999999999996E-2</v>
       </c>
       <c r="R11" s="11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>4.0000000000000001E-3</v>
       </c>
       <c r="S11" s="11"/>
@@ -1862,17 +1928,17 @@
         <v>27</v>
       </c>
       <c r="N12" s="6" t="b">
-        <f>I12&gt;H12</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O12" s="6" t="b">
-        <f>I12&gt;J12</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P12" s="6"/>
       <c r="Q12" s="6"/>
       <c r="R12" s="11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2.3800000000000004E-4</v>
       </c>
       <c r="S12" s="11"/>
@@ -1914,17 +1980,17 @@
         <v>45</v>
       </c>
       <c r="N13" s="6" t="b">
-        <f>I13&gt;H13</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O13" s="6" t="b">
-        <f>I13&gt;J13</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P13" s="6"/>
       <c r="Q13" s="6"/>
       <c r="R13" s="11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S13" s="11"/>
@@ -1967,23 +2033,23 @@
         <v>30</v>
       </c>
       <c r="N14" s="6" t="b">
-        <f>I14&gt;H14</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O14" s="6" t="b">
-        <f>I14&gt;J14</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P14" s="11">
-        <f t="shared" ref="P14" si="5">H14*3600*24</f>
+        <f t="shared" ref="P14" si="7">H14*3600*24</f>
         <v>2E-3</v>
       </c>
       <c r="Q14" s="11">
-        <f t="shared" ref="Q14" si="6">I14*3600*24</f>
+        <f t="shared" ref="Q14" si="8">I14*3600*24</f>
         <v>0.04</v>
       </c>
       <c r="R14" s="11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2.6999999999999996E-2</v>
       </c>
       <c r="S14" s="11"/>
@@ -2027,13 +2093,13 @@
         <v>1</v>
       </c>
       <c r="O15" s="6" t="b">
-        <f>I15&gt;J15</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P15" s="6"/>
       <c r="Q15" s="6"/>
       <c r="R15" s="11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2.3328000000000003E-3</v>
       </c>
       <c r="S15" s="11"/>
@@ -2069,17 +2135,17 @@
         <v>20</v>
       </c>
       <c r="N16" s="6" t="b">
-        <f>I16&gt;H16</f>
+        <f t="shared" ref="N16:N26" si="9">I16&gt;H16</f>
         <v>1</v>
       </c>
       <c r="O16" s="6" t="b">
-        <f>I16&gt;J16</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P16" s="6"/>
       <c r="Q16" s="6"/>
       <c r="R16" s="11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S16" s="11"/>
@@ -2113,11 +2179,11 @@
         <v>20</v>
       </c>
       <c r="N17" s="6" t="b">
-        <f>I17&gt;H17</f>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="O17" s="6" t="b">
-        <f>I17&gt;J17</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P17" s="6"/>
@@ -2167,17 +2233,17 @@
         <v>27</v>
       </c>
       <c r="N18" s="6" t="b">
-        <f>I18&gt;H18</f>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="O18" s="6" t="b">
-        <f>I18&gt;J18</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P18" s="6"/>
       <c r="Q18" s="6"/>
       <c r="R18" s="11">
-        <f t="shared" ref="R18" si="7">J18*3600*24</f>
+        <f t="shared" ref="R18" si="10">J18*3600*24</f>
         <v>2.3800000000000004E-4</v>
       </c>
       <c r="S18" s="11"/>
@@ -2214,11 +2280,11 @@
         <v>20</v>
       </c>
       <c r="N19" s="6" t="b">
-        <f>I19&gt;H19</f>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="O19" s="6" t="b">
-        <f>I19&gt;J19</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P19" s="6"/>
@@ -2258,11 +2324,11 @@
         <v>20</v>
       </c>
       <c r="N20" s="6" t="b">
-        <f>I20&gt;H20</f>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="O20" s="6" t="b">
-        <f>I20&gt;J20</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P20" s="6"/>
@@ -2307,17 +2373,17 @@
         <v>45</v>
       </c>
       <c r="N21" s="6" t="b">
-        <f>I21&gt;H21</f>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="O21" s="6" t="b">
-        <f>I21&gt;J21</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P21" s="6"/>
       <c r="Q21" s="6"/>
       <c r="R21" s="11">
-        <f t="shared" ref="R21:R26" si="8">J21*3600*24</f>
+        <f t="shared" ref="R21:R26" si="11">J21*3600*24</f>
         <v>0</v>
       </c>
       <c r="S21" s="11"/>
@@ -2360,23 +2426,23 @@
         <v>32</v>
       </c>
       <c r="N22" s="6" t="b">
-        <f>I22&gt;H22</f>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="O22" s="6" t="b">
-        <f>I22&gt;J22</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P22" s="11">
-        <f t="shared" ref="P22" si="9">H22*3600*24</f>
+        <f t="shared" ref="P22" si="12">H22*3600*24</f>
         <v>8.6400000000000004E-16</v>
       </c>
       <c r="Q22" s="11">
-        <f t="shared" ref="Q22" si="10">I22*3600*24</f>
+        <f t="shared" ref="Q22" si="13">I22*3600*24</f>
         <v>5.5484999999999995E-5</v>
       </c>
       <c r="R22" s="11">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>2.5000000000000001E-5</v>
       </c>
       <c r="S22" s="11"/>
@@ -2423,17 +2489,17 @@
         <v>27</v>
       </c>
       <c r="N23" s="6" t="b">
-        <f>I23&gt;H23</f>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="O23" s="6" t="b">
-        <f>I23&gt;J23</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P23" s="6"/>
       <c r="Q23" s="6"/>
       <c r="R23" s="11">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>2.3800000000000004E-4</v>
       </c>
       <c r="S23" s="11"/>
@@ -2475,17 +2541,17 @@
         <v>45</v>
       </c>
       <c r="N24" s="6" t="b">
-        <f>I24&gt;H24</f>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="O24" s="6" t="b">
-        <f>I24&gt;J24</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P24" s="6"/>
       <c r="Q24" s="6"/>
       <c r="R24" s="11">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="S24" s="11"/>
@@ -2530,23 +2596,23 @@
         <v>32</v>
       </c>
       <c r="N25" s="6" t="b">
-        <f>I25&gt;H25</f>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="O25" s="6" t="b">
-        <f>I25&gt;J25</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P25" s="11">
-        <f t="shared" ref="P25:P26" si="11">H25*3600*24</f>
+        <f t="shared" ref="P25:P26" si="14">H25*3600*24</f>
         <v>8.6400000000000004E-16</v>
       </c>
       <c r="Q25" s="11">
-        <f t="shared" ref="Q25:Q26" si="12">I25*3600*24</f>
+        <f t="shared" ref="Q25:Q26" si="15">I25*3600*24</f>
         <v>5.5484999999999996E-4</v>
       </c>
       <c r="R25" s="11">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>2.5000000000000001E-4</v>
       </c>
       <c r="S25" s="11"/>
@@ -2590,23 +2656,23 @@
         <v>37</v>
       </c>
       <c r="N26" s="6" t="b">
-        <f>I26&gt;H26</f>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="O26" s="6" t="b">
-        <f>I26&gt;J26</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P26" s="11">
+        <f t="shared" si="14"/>
+        <v>8.6400000000000004E-16</v>
+      </c>
+      <c r="Q26" s="11">
+        <f t="shared" si="15"/>
+        <v>2.5919999999999999E-6</v>
+      </c>
+      <c r="R26" s="11">
         <f t="shared" si="11"/>
-        <v>8.6400000000000004E-16</v>
-      </c>
-      <c r="Q26" s="11">
-        <f t="shared" si="12"/>
-        <v>2.5919999999999999E-6</v>
-      </c>
-      <c r="R26" s="11">
-        <f t="shared" si="8"/>
         <v>1.7712000000000001E-6</v>
       </c>
       <c r="S26" s="11"/>
@@ -2638,7 +2704,7 @@
         <v>50</v>
       </c>
       <c r="N27" s="6" t="b">
-        <f t="shared" ref="N16:N60" si="13">I27&gt;H27</f>
+        <f t="shared" ref="N27:N60" si="16">I27&gt;H27</f>
         <v>1</v>
       </c>
       <c r="O27" s="6" t="b">
@@ -2675,7 +2741,7 @@
         <v>50</v>
       </c>
       <c r="N28" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O28" s="6" t="b">
@@ -2709,7 +2775,7 @@
         <v>50</v>
       </c>
       <c r="N29" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O29" s="6" t="b">
@@ -2729,7 +2795,7 @@
       <c r="G30" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="H30" s="48">
+      <c r="H30" s="25">
         <v>0.5</v>
       </c>
       <c r="I30" s="25">
@@ -2743,7 +2809,7 @@
         <v>50</v>
       </c>
       <c r="N30" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O30" s="6" t="b">
@@ -2777,7 +2843,7 @@
         <v>50</v>
       </c>
       <c r="N31" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O31" s="6" t="b">
@@ -2812,7 +2878,7 @@
         <v>57</v>
       </c>
       <c r="N32" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O32" s="6" t="b">
@@ -2849,7 +2915,7 @@
         <v>50</v>
       </c>
       <c r="N33" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O33" s="6" t="b">
@@ -2886,11 +2952,11 @@
         <v>50</v>
       </c>
       <c r="N34" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O34" s="6" t="b">
-        <f t="shared" ref="O34:O60" si="14">I34&gt;J34</f>
+        <f t="shared" ref="O34:O60" si="17">I34&gt;J34</f>
         <v>1</v>
       </c>
       <c r="P34" s="6"/>
@@ -2920,11 +2986,11 @@
         <v>50</v>
       </c>
       <c r="N35" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O35" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P35" s="6"/>
@@ -2951,11 +3017,11 @@
         <v>63</v>
       </c>
       <c r="N36" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O36" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P36" s="6"/>
@@ -2988,11 +3054,11 @@
         <v>50</v>
       </c>
       <c r="N37" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O37" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P37" s="6"/>
@@ -3008,7 +3074,7 @@
       <c r="G38" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="H38" s="48">
+      <c r="H38" s="25">
         <v>0.15</v>
       </c>
       <c r="I38" s="25">
@@ -3022,11 +3088,11 @@
         <v>50</v>
       </c>
       <c r="N38" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O38" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P38" s="6"/>
@@ -3053,11 +3119,11 @@
         <v>63</v>
       </c>
       <c r="N39" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O39" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P39" s="6"/>
@@ -3087,11 +3153,11 @@
         <v>49</v>
       </c>
       <c r="N40" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O40" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P40" s="6"/>
@@ -3118,11 +3184,11 @@
         <v>63</v>
       </c>
       <c r="N41" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O41" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P41" s="6"/>
@@ -3154,11 +3220,11 @@
         <v>72</v>
       </c>
       <c r="N42" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="O42" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="P42" s="6"/>
@@ -3190,11 +3256,11 @@
         <v>72</v>
       </c>
       <c r="N43" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="O43" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="P43" s="6"/>
@@ -3226,11 +3292,11 @@
         <v>76</v>
       </c>
       <c r="N44" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O44" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P44" s="6"/>
@@ -3261,11 +3327,11 @@
         <v>76</v>
       </c>
       <c r="N45" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O45" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P45" s="6"/>
@@ -3296,11 +3362,11 @@
         <v>76</v>
       </c>
       <c r="N46" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O46" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P46" s="6"/>
@@ -3331,11 +3397,11 @@
         <v>76</v>
       </c>
       <c r="N47" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O47" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P47" s="6"/>
@@ -3366,11 +3432,11 @@
         <v>76</v>
       </c>
       <c r="N48" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O48" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P48" s="6"/>
@@ -3398,11 +3464,11 @@
         <v>77</v>
       </c>
       <c r="N49" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O49" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P49" s="6"/>
@@ -3434,11 +3500,11 @@
         <v>79</v>
       </c>
       <c r="N50" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O50" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P50" s="6"/>
@@ -3469,11 +3535,11 @@
         <v>76</v>
       </c>
       <c r="N51" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O51" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P51" s="6"/>
@@ -3504,11 +3570,11 @@
         <v>80</v>
       </c>
       <c r="N52" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O52" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P52" s="6"/>
@@ -3542,11 +3608,11 @@
         <v>76</v>
       </c>
       <c r="N53" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O53" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P53" s="6"/>
@@ -3577,11 +3643,11 @@
         <v>79</v>
       </c>
       <c r="N54" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O54" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P54" s="6"/>
@@ -3615,11 +3681,11 @@
         <v>79</v>
       </c>
       <c r="N55" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O55" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P55" s="6"/>
@@ -3650,11 +3716,11 @@
         <v>75</v>
       </c>
       <c r="N56" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O56" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P56" s="6"/>
@@ -3686,11 +3752,11 @@
         <v>85</v>
       </c>
       <c r="N57" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O57" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P57" s="6"/>
@@ -3727,11 +3793,11 @@
         <v>85</v>
       </c>
       <c r="N58" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O58" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P58" s="6"/>
@@ -3768,11 +3834,11 @@
         <v>85</v>
       </c>
       <c r="N59" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O59" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P59" s="6"/>
@@ -3806,11 +3872,11 @@
         <v>87</v>
       </c>
       <c r="N60" s="6" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O60" s="6" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="P60" s="6"/>
@@ -3979,9 +4045,9 @@
       <c r="B2" t="s">
         <v>92</v>
       </c>
-      <c r="D2" t="e">
-        <f>#REF!*1000000</f>
-        <v>#REF!</v>
+      <c r="D2">
+        <f>'[1]Netherlands scale calculations'!B4*1000000</f>
+        <v>41543000000</v>
       </c>
       <c r="E2" t="s">
         <v>93</v>
@@ -3995,13 +4061,13 @@
       <c r="B3" t="s">
         <v>92</v>
       </c>
-      <c r="D3" s="25" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="G3" t="e">
+      <c r="D3" s="25">
+        <f>'[1]Netherlands scale calculations'!C2</f>
+        <v>9.9944635678694368E-2</v>
+      </c>
+      <c r="G3">
         <f>D2*D3</f>
-        <v>#REF!</v>
+        <v>4152000000</v>
       </c>
       <c r="N3" s="30"/>
     </row>
@@ -4015,13 +4081,13 @@
       <c r="C4" t="s">
         <v>96</v>
       </c>
-      <c r="D4" s="30" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="G4" t="e">
+      <c r="D4" s="30">
+        <f>'[1]Netherlands scale calculations'!H2</f>
+        <v>0.5965071808724024</v>
+      </c>
+      <c r="G4">
         <f>($D$2-$G$3)*D4</f>
-        <v>#REF!</v>
+        <v>22303999999.999996</v>
       </c>
       <c r="N4" s="30"/>
     </row>
@@ -4035,13 +4101,13 @@
       <c r="C5" t="s">
         <v>97</v>
       </c>
-      <c r="D5" s="30" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="G5" t="e">
+      <c r="D5" s="30">
+        <f>'[1]Netherlands scale calculations'!H3</f>
+        <v>5.3060897007301225E-2</v>
+      </c>
+      <c r="G5">
         <f>($D$2-$G$3)*D5</f>
-        <v>#REF!</v>
+        <v>1984000000</v>
       </c>
       <c r="N5" s="30"/>
     </row>
@@ -4055,13 +4121,13 @@
       <c r="C6" t="s">
         <v>98</v>
       </c>
-      <c r="D6" s="30" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="G6" t="e">
+      <c r="D6" s="30">
+        <f>'[1]Netherlands scale calculations'!H4</f>
+        <v>0.13412318472359658</v>
+      </c>
+      <c r="G6">
         <f>($D$2-$G$3)*D6</f>
-        <v>#REF!</v>
+        <v>5015000000</v>
       </c>
       <c r="N6" s="30"/>
     </row>
@@ -4075,13 +4141,13 @@
       <c r="C7" t="s">
         <v>99</v>
       </c>
-      <c r="D7" s="30" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="G7" t="e">
+      <c r="D7" s="30">
+        <f>'[1]Netherlands scale calculations'!H5</f>
+        <v>0.16923858682570672</v>
+      </c>
+      <c r="G7">
         <f>($D$2-$G$3)*D7</f>
-        <v>#REF!</v>
+        <v>6328000000</v>
       </c>
       <c r="M7" s="29"/>
     </row>
@@ -4095,13 +4161,13 @@
       <c r="C8" t="s">
         <v>100</v>
       </c>
-      <c r="D8" s="30" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="G8" t="e">
+      <c r="D8" s="30">
+        <f>'[1]Netherlands scale calculations'!H6</f>
+        <v>4.7070150570993022E-2</v>
+      </c>
+      <c r="G8">
         <f>($D$2-$G$3)*D8</f>
-        <v>#REF!</v>
+        <v>1760000000</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
@@ -4709,6 +4775,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0577e6a0-5f74-4659-a81a-c7bdc984432d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="f5c8fe0e-f8db-4fac-9fd3-e69469f9c90b" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FF634CA3F5682C418397C6E4414BCDE3" ma:contentTypeVersion="19" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="cd864e38cd6bbc6c7e0427721adcc1d0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="0577e6a0-5f74-4659-a81a-c7bdc984432d" xmlns:ns3="f5c8fe0e-f8db-4fac-9fd3-e69469f9c90b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fa37df3857ed3652683061e5b337c961" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -4974,36 +5062,42 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0577e6a0-5f74-4659-a81a-c7bdc984432d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="f5c8fe0e-f8db-4fac-9fd3-e69469f9c90b" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D108A85F-60BE-4139-A6D5-7B3D23DBFDB3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9DFF8A43-35D3-4DC9-B58B-6B849DF01427}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0577e6a0-5f74-4659-a81a-c7bdc984432d"/>
+    <ds:schemaRef ds:uri="f5c8fe0e-f8db-4fac-9fd3-e69469f9c90b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80C5A0E2-4FC7-4E62-829B-76F1D157D51F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80C5A0E2-4FC7-4E62-829B-76F1D157D51F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9DFF8A43-35D3-4DC9-B58B-6B849DF01427}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D108A85F-60BE-4139-A6D5-7B3D23DBFDB3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="0577e6a0-5f74-4659-a81a-c7bdc984432d"/>
+    <ds:schemaRef ds:uri="f5c8fe0e-f8db-4fac-9fd3-e69469f9c90b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>